<commit_message>
Mise à jour du vocabulaires avec celui du Semic + tout le vocabulaire sur schema.data.gouv.fr outre que les pdfs (que les standards qui ont une modélisation uml) et mise a jour du prompt pour prendre automatiquement le vocabulaire et la description dans vocabularies.xlsx
</commit_message>
<xml_diff>
--- a/tools/index_search/vocabularies.xlsx
+++ b/tools/index_search/vocabularies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gglesner001\Documents\GitHub\AI4semantics\tools\index_search\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\theojoly\AI4Semantics\AI4Semantics-MCP-server-fr\tools\index_search\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5ECBC1F-2F92-483F-914E-3ECB39B46D93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2502459A-B6A7-4D2E-B130-5B9BB4100F4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30720" yWindow="-29220" windowWidth="16440" windowHeight="28320" xr2:uid="{0A5BC981-4B30-4287-845A-45F617C3BDE0}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0A5BC981-4B30-4287-845A-45F617C3BDE0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,16 +27,17 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="148">
   <si>
     <t>CBV</t>
   </si>
@@ -95,12 +96,6 @@
     <t>The Core Public Service Vocabulary Application Profile (CPSV-AP) is a reusable and extensible data specification used for harmonising the way public services are described in a machine-readable format. CPSV-AP captures fundamental characteristics of a public service, such as the name, description, competent public organisation, output, etc. Public administrations and service providers can therefore use this approach to describe their services and guarantee a level of cross-domain and cross-border interoperability at European, national and local level.</t>
   </si>
   <si>
-    <t>OSLO_Organisatie</t>
-  </si>
-  <si>
-    <t>OSLO_Persoon</t>
-  </si>
-  <si>
     <t>NAME</t>
   </si>
   <si>
@@ -111,41 +106,407 @@
 This specification enables interoperability among registers and any other ICT based solutions exchanging and processing person-related information.</t>
   </si>
   <si>
-    <t>OSLO_Adres</t>
-  </si>
-  <si>
-    <t>OSLO-Persoon richt zich op het beschrijven van een natuurlijk persoon, d.w.z. een fysiek persoon en geen organisatie. Natuurlijke personen hebben een eigen rechtspersoonlijkheid, deze is niet kunstmatig zoals bij rechtspersonen.</t>
-  </si>
-  <si>
-    <t>Het vocabularium Observaties en Metingen bevat de terminologie nodig om Observaties te beschrijven.</t>
-  </si>
-  <si>
-    <t>OSLO_Gebouw</t>
-  </si>
-  <si>
-    <t>Het OSLO-Adres vocabularium voegt termen toe aan bestaande RDF-vocabularia zodat gestructureerde adressen kunnen worden uitgewisseld. Een Europese standaard voor dergelijke adressen bestaat (INSPIRE-Address) maar heeft momenteel nog geen RDF-vocabularium. Bovendien is deze standaard bedoeld om om het even welk Europees adres te beschrijven, hij is m.a.w. te generiek voor uitwisseling van Belgische adressen. We zorgden er echter voor dat OSLO-Adres perfect mapt op INSPIRE-Address.</t>
-  </si>
-  <si>
-    <t>OSLO-Organisatie voegt termen toe aan drie bestaande vocabularia waarmee organisaties worden beschreven.</t>
-  </si>
-  <si>
-    <t>Het vocabularium OSLO-Gebouw focust op termen die betrekking hebben op gebouwen en gebouweenheden. Vertrekpunt vormden termen gedefinieerd voor deze entiteiten in het Gebouwenregister (VBR). Echter gebeurde ook afstemming met INSPIRE-Building en met de federale werkgroep rond gebouwen (GT-BUNI).</t>
-  </si>
-  <si>
-    <t>OSLO_Observaties_en_Metingen</t>
-  </si>
-  <si>
     <t>CAV</t>
   </si>
   <si>
     <t>The Core Assessment Vocabulary represents, expresses, and defines what an “Assessment” of “Assets” is and how to perform the assessment based on “Criteria”. It is a domain-agnostic vocabulary, meaning that it can be used to assess any asset. The CAV addresses semantic interoperability by reusing existing generic ontologies and vocabularies. This way, the semantics of common concepts and properties are agreed without having to re-discuss them. When concepts or properties have not been identified nor defined for the purposes pursued, they have to be proposed either as extensions or from scratch.</t>
+  </si>
+  <si>
+    <t>SDG-AC</t>
+  </si>
+  <si>
+    <t>Arrêtés permanents de circulation pour le transport de marchandises. Spécification du fichier d'échange relatif aux arrêtés permanents de circulation pour le transport de marchandises gérés par les collectivités.</t>
+  </si>
+  <si>
+    <t>SDG-ACM</t>
+  </si>
+  <si>
+    <t>Aménagement cyclable. Spécification du fichier d'échange relatif aux données concernant la localisation géographique et les caractéristiques des aménagements cyclables</t>
+  </si>
+  <si>
+    <t>Ce modèle structure les données d’accessibilité des ERP autour de l’établissement, de ses entrées et des cheminements entre celles-ci, en décrivant leurs caractéristiques (accueil, stationnement, équipements, pentes, obstacles) afin d’évaluer la facilité d’accès pour tous.</t>
+  </si>
+  <si>
+    <t>SDG-AERP</t>
+  </si>
+  <si>
+    <t>Aires de livraison. Spécification du fichier d'échange relatif aux aires de livraison.</t>
+  </si>
+  <si>
+    <t>SDG-AL</t>
+  </si>
+  <si>
+    <t>Atlas Paysager. Un atlas du paysage est un document de connaissance des paysages. Cette classe est destinée à fournir à l’utilisateur des informations générales sur l’atlas, ses conditions de réalisation et de mise à jour.</t>
+  </si>
+  <si>
+    <t>SDG-AP</t>
+  </si>
+  <si>
+    <t>Ce modèle décrit l’accessibilité de la voirie en reliant les cheminements, les tronçons, les nœuds, les obstacles et les équipements d’accès, afin de caractériser les parcours et leurs contraintes.</t>
+  </si>
+  <si>
+    <t>SDG-AV</t>
+  </si>
+  <si>
+    <t>Base Adresse Locale v1.5. Spécification du fichier d'échange visant à diffuser des données voies-adresses locales.</t>
+  </si>
+  <si>
+    <t>SDG-BS</t>
+  </si>
+  <si>
+    <t>Budget des collectivités et établissements publics locaux. Les données essentielles du budget permettent de décrire le contenu des étapes budgétaires des collectivités locales et des établissements publics. Il permet de préciser les catégories de montants financiers ainsi que le découpage de ces sommes en fonction du type de présentation utilisé (par nature ou par fonction). Ce schéma décrit le détail de chaque champ et le cas échéant les règles de validité associées.</t>
+  </si>
+  <si>
+    <t>SDG-BUDG</t>
+  </si>
+  <si>
+    <t>Catalogue simplifié. Spécification du modèle de données relatif au catalogue des jeux de données publiés en open data par une collectivité.</t>
+  </si>
+  <si>
+    <t>SDG-CATAL</t>
+  </si>
+  <si>
+    <t>Déclaration de l'acquisition de biens issus du réemploi, de la réutilisation ou intégrant des matières recyclées. Spécification du fichier d'échange relatif aux déclarations de la part des dépenses relatives à l'acquisition de biens issus du réemploi ou de la réutilisation ou intégrant des matières recyclées (loi AGEC).</t>
+  </si>
+  <si>
+    <t>SDG-CDBRRC</t>
+  </si>
+  <si>
+    <t>Comptage des mobilités (Channel). Spécification du fichier d'échange relatif aux comptages des mobilités.</t>
+  </si>
+  <si>
+    <t>SDG-CMC</t>
+  </si>
+  <si>
+    <t>Comptage des mobilités (Measure). Spécification du fichier d'échange relatif aux comptages des mobilités.</t>
+  </si>
+  <si>
+    <t>SDG-CMM</t>
+  </si>
+  <si>
+    <t>Collectivités. Schéma de données pour décrire les collectivités territoriales associées aux projets de transition écologique.</t>
+  </si>
+  <si>
+    <t>SDG-COLL</t>
+  </si>
+  <si>
+    <t>DAE. Spécification du modèle de données relatif aux DAE.</t>
+  </si>
+  <si>
+    <t>SDG-DAE</t>
+  </si>
+  <si>
+    <t>Format réglementaire de publication des données essentielles des marchés publics français.</t>
+  </si>
+  <si>
+    <t>SDG-DECP</t>
+  </si>
+  <si>
+    <t>Délibérations. Spécification du modèle de données relatif aux délibérations adoptées par une collectivité locale.</t>
+  </si>
+  <si>
+    <t>SDG-DELIB</t>
+  </si>
+  <si>
+    <t>Dispositifs d'aides. Spécification du fichier d'échange relatif aux dispositifs d'aides.</t>
+  </si>
+  <si>
+    <t>SDG-DISAI</t>
+  </si>
+  <si>
+    <t>Document Paysage. Un document paysage est un document illustrant un découpage paysager. Il peut s’agir d’un bloc-diagramme, d’une coupe, d’un croquis, d’une photographie, etc.</t>
+  </si>
+  <si>
+    <t>SDG-DOCP</t>
+  </si>
+  <si>
+    <t>Schéma des données d'accessibilité des ERPs. Spécification du fichier d'échange relatif aux données d'accessibilité des Établissements Recevant du Public (ERP).</t>
+  </si>
+  <si>
+    <t>SDG-DONNA</t>
+  </si>
+  <si>
+    <t>Dynamique. Une dynamique est une évolution du paysage en général depuis la dernière version de l’atlas des paysages.\nUne dynamique est modélisée par un « data type », c’est-à-dire un attribut complexe ; celui-ci peut s’appliquer à tout niveau de découpage paysager : sous-unités paysagères, unités paysagères, ensembles paysagers.\nUn découpage paysager peut avoir plusieurs dynamiques.</t>
+  </si>
+  <si>
+    <t>SDG-DYNA</t>
+  </si>
+  <si>
+    <t>Ce modèle détaille les équipements d'accès (traversées, rampes, escaliers, ascenseurs, élévateurs, escalators, tapis roulants, entrées, passages sélectifs, quais) avec leurs caractéristiques techniques pour évaluer leur accessibilité.</t>
+  </si>
+  <si>
+    <t>SDG-EA</t>
+  </si>
+  <si>
+    <t>Ensemble Paysager. Un ensemble paysager est observé à l’échelle d’un territoire régional. Il est issu de l’association de plusieurs unités paysagères dont les caracté-istiques géomorphologiques, écologiques, d’occupation du sol et de perception des habitants et des acteurs sont cohérentes à l’échelle dézoomée du territoire régional. Comme pour les unités paysagères, les limites entre ensembles paysagers peuvent être nettes ou « floues ». Cette nomination « EP » englobe celles parfois usitées telles que « grands paysages », « grands ensembles paysagers », « grandes entités paysagères », etc.</t>
+  </si>
+  <si>
+    <t>SDG-ENSPAY</t>
+  </si>
+  <si>
+    <t>Équipements. Spécification du modèle de données relatif aux équipements collectifs publics d'une collectivité.</t>
+  </si>
+  <si>
+    <t>SDG-EQUIP</t>
+  </si>
+  <si>
+    <t>Schéma des fontaines à eau. Spécification du fichier d'échange relatif aux fontaines à eau mises à disposition notamment par les Etablissements recevant du public (ERP) dans le cadre de la loi anti-gaspillage.</t>
+  </si>
+  <si>
+    <t>SDG-FONTEA</t>
+  </si>
+  <si>
+    <t>Standard CNIG Friches. Spécification du fichier d'échange conforme au standard CNIG Friches relatif aux friches urbanisées. Une friche \"urbanisée\" a connu une activité économique (industrielle, artisanale, logistique, commerciale, de loisir, tertiaire, agricole), un usage résidentiel ou un usage d'équipement. La définition règlementaire décrit \"tout bien ou droit immobilier, bâti ou non bâti, inutilisé et dont l'état, la configuration ou l'occupation totale ou partielle ne permet pas un réemploi sans un aménagement ou des travaux préalables\". En particulier, les friches dites \"agricoles\", au sens des espaces auparavant cultivés et qui se sont enfrichés, ne sont pas prises en compte dans le cadre de ce standard, au contraire des bâtis agricoles désaffectés.</t>
+  </si>
+  <si>
+    <t>SDG-FRI</t>
+  </si>
+  <si>
+    <t>Hautes rémunérations dans la fonction publique. Spécification du fichier de déclaration des dix rémunérations les plus élevées des agents publiques.</t>
+  </si>
+  <si>
+    <t>SDG-HR</t>
+  </si>
+  <si>
+    <t>Indice de durabilité - Lave-linge. Schéma de données pour l'indice de durabilité - lave-linge.</t>
+  </si>
+  <si>
+    <t>Indice de durabilité - Téléviseur. Schéma de données pour l'indice de durabilité - téléviseur.</t>
+  </si>
+  <si>
+    <t>SDG-IDT</t>
+  </si>
+  <si>
+    <t>SDG-IDLL</t>
+  </si>
+  <si>
+    <t>IRVE dynamique. Spécification du fichier d'échange relatif aux données concernant l’état temps réel des points de recharge pour véhicules électriques. Chaque ligne du fichier correspond à un point de recharge (PDC) dont les caractéristiques complètes sont décrites dans un fichier au schéma « IRVE statique ».</t>
+  </si>
+  <si>
+    <t>SDG-IDYN</t>
+  </si>
+  <si>
+    <t>Indice de réparabilité. Schéma de données pour l'indice de réparabilité.</t>
+  </si>
+  <si>
+    <t>SDG-IR</t>
+  </si>
+  <si>
+    <t>Itinéraires de randonnée. Spécification du fichier d'échange relatif aux itinéraires de randonnée.</t>
+  </si>
+  <si>
+    <t>SDG-IRA</t>
+  </si>
+  <si>
+    <t>Impact d’un service public numérique. Schéma de données pour les indicateurs d’impact d’un service public numérique.</t>
+  </si>
+  <si>
+    <t>SDG-ISPN</t>
+  </si>
+  <si>
+    <t>IRVE statique. Spécification du fichier d'échange relatif aux données concernant la localisation géographique et les caractéristiques techniques des stations et des points de recharge pour véhicules électriques. Chaque ligne du fichier correspond à un point de recharge (PDC).</t>
+  </si>
+  <si>
+    <t>SDG-ISTAT</t>
+  </si>
+  <si>
+    <t>Informations travaux. L'[article L49](https://www.legifrance.gouv.fr/affichCodeArticle.do?cidTexte=LEGITEXT000006070987&amp;idArticle=LEGIARTI000021493642) du code des postes et des communications électroniques a introduit le devoir de publicité de travaux d'infrastructures. Le schéma **Informations travaux** s'inscrit dans la continuité de cette réglementation avec l'objectif de simplifier et standardiser le partage de cette information afin de maximiser les externalités positives qui découlent de l'anticipation des travaux de génie civil.</t>
+  </si>
+  <si>
+    <t>SDG-IT</t>
+  </si>
+  <si>
+    <t>Lieux de covoiturage. Spécification des lieux permettant le covoiturage.</t>
+  </si>
+  <si>
+    <t>SDG-LC</t>
+  </si>
+  <si>
+    <t>SDG-LDP</t>
+  </si>
+  <si>
+    <t>Lieux de stationnement. Spécification des lieux permettant le stationnement en parc.</t>
+  </si>
+  <si>
+    <t>SDG-LSTAT</t>
+  </si>
+  <si>
+    <t>Menus de la restauration collective. Schéma permettant de décrire les menus des repas proposés par les collectivités locales, les établissements publics et privés. Il permet de préciser les modalités de distribution et le contenu des menus proposés (les plats). Le choix a été fait de détailler chaque plat sur une ligne. Pour décrire un menu il faut donc répéter certaines informations plusieurs fois.</t>
+  </si>
+  <si>
+    <t>Limite Découpage Paysager. Une limite de découpage paysager est une portion du contour d’un découpage paysager : unité paysagère ou ensemble paysager ou sous-ensemble paysager.Cette classe est essentiellement destinée à renseigner l’utilisateur sur la nature et la précision de la limite.</t>
+  </si>
+  <si>
+    <t>SDG-MCOL</t>
+  </si>
+  <si>
+    <t>Classe OPERATION-AMENAGEMENT du standard CNIG Opérations d'aménagement. Spécification du fichier d'échange conforme au standard CNIG Opérations d'aménagement pour la classe OPERATION-AMENAGEMENT.</t>
+  </si>
+  <si>
+    <t>SDG-OA</t>
+  </si>
+  <si>
+    <t>SDG-OINS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onstreet parking reprensentation. </t>
+  </si>
+  <si>
+    <t>SDG-ONP</t>
+  </si>
+  <si>
+    <t>Offre d'insertion. Ce schéma JSON structure les services d'inclusion en définissant leurs attributs d'identification, de localisation, de contact, leurs caractéristiques (type, thématiques, publics), modalités d'accès (frais, modes d'accueil, mobilisation) et informations temporelles (durée, horaires).</t>
+  </si>
+  <si>
+    <t>Schéma pour les passages à niveau. Spécification du fichier décrivant les emplacements de passages à niveau.</t>
+  </si>
+  <si>
+    <t>SDG-PASSN</t>
+  </si>
+  <si>
+    <t>Point d'Eau Incendie (PEI). Spécification du modèle de données relatif aux PEI.</t>
+  </si>
+  <si>
+    <t>SDG-PEI</t>
+  </si>
+  <si>
+    <t>Composition des plats des menus de la restauration collective. Description des plats proposés par des collectivités locales, des établissements publics et des entreprises dans le cadre de l'offre de restauration collective. Il permet de préciser les modalités de fabrication des plats et de détailler les produits qui les composent. Ce schéma décrit le détail de chaque champ et le cas échéant les règles de validité associées. Il peut être utilisé indépendamment ou en complément du le schéma sur les menus collectifs qui décrit la composition en plats.</t>
+  </si>
+  <si>
+    <t>SDG-PMCOLL</t>
+  </si>
+  <si>
+    <t>Prénoms des nouveaux-nés. Spécification du modèle de données relatif aux prénoms des nouveaux-nés déclarés à l’état-civil.</t>
+  </si>
+  <si>
+    <t>SDG-PNN</t>
+  </si>
+  <si>
+    <t>Classe PROGRAMME du standard CNIG Opérations d'aménagement. Spécification du fichier d'échange conforme au standard CNIG Opérations d'aménagement pour la classe PROGRAMME.</t>
+  </si>
+  <si>
+    <t>SDG-PROG</t>
+  </si>
+  <si>
+    <t>Projets de collectivités. Schéma de données pour décrire un projet de collectivité visant la transition écologique, incluant les informations de suivi, le budget, le statut, les détails du porteur et les référentiels de compétences et leviers.</t>
+  </si>
+  <si>
+    <t>SDG-PTER</t>
+  </si>
+  <si>
+    <t>Registre d'entrée d'archives. Spécification du standard national des registres d'entrée d'archives.</t>
+  </si>
+  <si>
+    <t>SDG-REA</t>
+  </si>
+  <si>
+    <t>Stationnement cyclable. Spécification du fichier décrivant les emplacements de stationnement cycable.</t>
+  </si>
+  <si>
+    <t>SDG-SC</t>
+  </si>
+  <si>
+    <t>Comptage des mobilités (Site). Spécification du fichier d'échange relatif aux comptages des mobilités.</t>
+  </si>
+  <si>
+    <t>SDG-SCMS</t>
+  </si>
+  <si>
+    <t>Schéma directeur des infrastructures de recharge pour véhicules électriques et hybrides rechargeables. Spécification du fichier d'échange relatif aux schéma directeur des infrastructures de recharge pour véhicules électriques et hybrides rechargeables.</t>
+  </si>
+  <si>
+    <t>SDG-SDIR</t>
+  </si>
+  <si>
+    <t>Classe SECTEUR du standard CNIG Opérations d'aménagement. Spécification du fichier d'échange conforme au standard CNIG Opérations d'aménagement pour la classe SECTEUR.</t>
+  </si>
+  <si>
+    <t>SDG-SECT</t>
+  </si>
+  <si>
+    <t>Classe ETABLISSEMENT du standard CNIG Sites Economiques. Spécification du fichier d'échange conforme au standard CNIG Sites Economiques pour la classe ETABLISSEMENT : établissement économique.</t>
+  </si>
+  <si>
+    <t>SDG-SEE</t>
+  </si>
+  <si>
+    <t>Classe POLE-ECO du standard CNIG Sites Economiques. Spécification du fichier d'échange conforme au standard CNIG Sites Economiques pour la classe POLE-ECO : Pôle économique.</t>
+  </si>
+  <si>
+    <t>SDG-SEPE</t>
+  </si>
+  <si>
+    <t>Classe SITE-ECO du standard CNIG Sites EconomiquesClasse SITE-ECO du standard CNIG Sites Economiques. Spécification du fichier d'échange conforme au standard CNIG Sites Economiques pour la classe SITE-ECO : Site économique.</t>
+  </si>
+  <si>
+    <t>SDG-SESE</t>
+  </si>
+  <si>
+    <t>Classe TERRAIN-ECO du standard CNIG Sites Economiques. Spécification du fichier d'échange conforme au standard CNIG Sites Economiques pour la classe TERRAIN-ECO : terrain économique.</t>
+  </si>
+  <si>
+    <t>SDG-SETE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spécification du fichier de déclaration de profil d'acheteur. </t>
+  </si>
+  <si>
+    <t>SDG-SFDPA</t>
+  </si>
+  <si>
+    <t>Lieux de médiation numérique. Spécification du standard national des lieux de médiation numérique.</t>
+  </si>
+  <si>
+    <t>SDG-SMN</t>
+  </si>
+  <si>
+    <t>Sous-unité Paysagère. Une sous-unité paysagère est une subdivision d’une unité paysagère. Le découpage y est réalisé de manière plus fine, les sous–unités présentant entre elles de légères variations des composantes paysagères (liées à la topographie, à la fonctionnalité des milieux, aux tissus urbains…). Les sous-unités sont particulièrement utilisées au sein des unités paysagères très urbaines et peuvent être compatibles avec un découpage par quartier. Comme pour les unités paysagères, les limites entre sous-unités peuvent être nettes ou « floues ».</t>
+  </si>
+  <si>
+    <t>SDG-SP</t>
+  </si>
+  <si>
+    <t>Stations de taxi. Spécification des stations de taxi à usage public.</t>
+  </si>
+  <si>
+    <t>SDG-ST</t>
+  </si>
+  <si>
+    <t>Subventions. Spécification du modèle de données relatif aux subventions attribuées par une collectivité.</t>
+  </si>
+  <si>
+    <t>SDG-SUBV</t>
+  </si>
+  <si>
+    <t>Unité Paysagère. L’unité paysagère est le découpage paysager central dans la construction de la connaissance du paysage, il est issu de la qualification et de la caractérisation des paysages à l’échelle globale du département. Elle désigne une partie continue de territoire homogène au regard de ses caractéristiques géomorphologiques, écologiques, d’occupation du sol et de perception que les habitants et acteurs du territoire lui portent. Ce « paysage donné » est caractérisé par un ensemble de structures paysagères et d’éléments de paysage qui lui procurent sa singularité.\nUne unité paysagère est distinguée des unités paysagères voisines par des limites qui peuvent être nettes ou « floues ».</t>
+  </si>
+  <si>
+    <t>SDG-UP</t>
+  </si>
+  <si>
+    <t>Part des véhicules à faibles émissions dans le renouvellement d'un parc. Spécification des données fixant les termes et modalités de publication du pourcentage de véhicules à faibles et à très faibles émissions parmi les véhicules intégrés dans un renouvellement de parc.</t>
+  </si>
+  <si>
+    <t>SDG-VFERP</t>
+  </si>
+  <si>
+    <t>Part des véhicules à faibles émissions dans le renouvellement des parcs d’entreprises de location, location-vente, de crédit-bail de véhicules, des plateformes de livraisons et des centrales de réservation de taxi et VTC. Spécification du fichier d’échange relatif aux parts de véhicules à faibles émissions dans les parcs de véhicules des entreprises de location, location-vente et crédit-bail de véhicules, des plateformes de livraison, des centrales de réservation de taxi et de VTC. Certaines données demandées nécessitent des champs qui doivent être transmis aux services de l'administration compétents, mais dont la publication sur data.gouv.fr n'est pas obligatoire.</t>
+  </si>
+  <si>
+    <t>SDG-VFERPS</t>
+  </si>
+  <si>
+    <t>Ce schéma GeoJSON structure les Zones à Faibles Émissions (ZFE) en définissant pour chaque zone ou tronçon les restrictions de circulation par type de véhicule (particuliers, utilitaires, poids lourds, autocars, deux-roues) selon les vignettes CRITAIR et les horaires d'application.</t>
+  </si>
+  <si>
+    <t>SDG-ZFE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -159,6 +520,12 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -182,13 +549,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -523,30 +893,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3554DC79-575A-4492-B1E0-587118B5E51E}">
-  <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B74"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="36.81640625" customWidth="1"/>
-    <col min="2" max="2" width="34.54296875" customWidth="1"/>
+    <col min="1" max="1" width="36.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" s="3" customFormat="1">
+      <c r="A2" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>26</v>
-      </c>
       <c r="B2" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="12.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="12.5" customHeight="1">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -554,7 +924,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="12.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" ht="12.5" customHeight="1">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -562,7 +932,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" ht="13.5" customHeight="1">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -570,7 +940,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" ht="13.5" customHeight="1">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -578,7 +948,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" ht="14" customHeight="1">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -586,7 +956,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" ht="13.5" customHeight="1">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -594,74 +964,536 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" ht="14" customHeight="1">
       <c r="A9" t="s">
         <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="15" customHeight="1">
       <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15" customHeight="1">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="15" customHeight="1">
+      <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="15" customHeight="1">
+      <c r="A13" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>18</v>
-      </c>
       <c r="B13" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="15" customHeight="1">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="1"/>
-    </row>
-    <row r="16" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="1"/>
-    </row>
-    <row r="17" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="1"/>
-    </row>
-    <row r="18" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="1"/>
-    </row>
-    <row r="19" spans="2:2" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="1"/>
-    </row>
-    <row r="20" spans="2:2" ht="12.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="1"/>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="14.5" customHeight="1">
+      <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="13.5" customHeight="1">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15" customHeight="1">
+      <c r="A17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15" customHeight="1">
+      <c r="A18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="14" customHeight="1">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="12.5" customHeight="1">
+      <c r="A20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="56">
+      <c r="A22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="28">
+      <c r="A23" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="42">
+      <c r="A24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="42">
+      <c r="A25" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="42">
+      <c r="A26" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="70">
+      <c r="A27" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="70">
+      <c r="A28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="154">
+      <c r="A29" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="84">
+      <c r="A30" t="s">
+        <v>59</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="238">
+      <c r="A31" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="42">
+      <c r="A32" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" t="s">
+        <v>65</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="280">
+      <c r="A34" t="s">
+        <v>67</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="56">
+      <c r="A35" t="s">
+        <v>69</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="42">
+      <c r="A36" t="s">
+        <v>73</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="42">
+      <c r="A37" t="s">
+        <v>72</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="112">
+      <c r="A38" t="s">
+        <v>75</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="28">
+      <c r="A39" t="s">
+        <v>77</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="42">
+      <c r="A40" t="s">
+        <v>79</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="42">
+      <c r="A41" t="s">
+        <v>81</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="98">
+      <c r="A42" t="s">
+        <v>83</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="210">
+      <c r="A43" t="s">
+        <v>85</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="28">
+      <c r="A44" t="s">
+        <v>87</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="112">
+      <c r="A45" t="s">
+        <v>88</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="28">
+      <c r="A46" t="s">
+        <v>90</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="140">
+      <c r="A47" t="s">
+        <v>93</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" ht="84">
+      <c r="A48" t="s">
+        <v>95</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" ht="112">
+      <c r="A49" t="s">
+        <v>96</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" t="s">
+        <v>98</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" ht="42">
+      <c r="A51" t="s">
+        <v>101</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="28">
+      <c r="A52" t="s">
+        <v>103</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="210">
+      <c r="A53" t="s">
+        <v>105</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="56">
+      <c r="A54" t="s">
+        <v>107</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" ht="84">
+      <c r="A55" t="s">
+        <v>109</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" ht="98">
+      <c r="A56" t="s">
+        <v>111</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" ht="42">
+      <c r="A57" t="s">
+        <v>113</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" ht="42">
+      <c r="A58" t="s">
+        <v>115</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" ht="42">
+      <c r="A59" t="s">
+        <v>117</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" ht="98">
+      <c r="A60" t="s">
+        <v>119</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" ht="84">
+      <c r="A61" t="s">
+        <v>121</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" ht="84">
+      <c r="A62" t="s">
+        <v>123</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" ht="70">
+      <c r="A63" t="s">
+        <v>125</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" ht="98">
+      <c r="A64" t="s">
+        <v>127</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" ht="84">
+      <c r="A65" t="s">
+        <v>129</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" ht="28">
+      <c r="A66" t="s">
+        <v>131</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" ht="42">
+      <c r="A67" t="s">
+        <v>133</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" ht="210">
+      <c r="A68" t="s">
+        <v>135</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" ht="28">
+      <c r="A69" t="s">
+        <v>137</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" ht="42">
+      <c r="A70" t="s">
+        <v>139</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" ht="266">
+      <c r="A71" t="s">
+        <v>141</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" ht="98">
+      <c r="A72" t="s">
+        <v>143</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" ht="252">
+      <c r="A73" t="s">
+        <v>145</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" ht="112">
+      <c r="A74" t="s">
+        <v>147</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>146</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>